<commit_message>
chore: prepare monorepo release
</commit_message>
<xml_diff>
--- a/docs/sources-a-telecharger-par-exercice-v2.xlsx
+++ b/docs/sources-a-telecharger-par-exercice-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Apps Pimms\ateliers-Bureautique\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44BF1B7-D093-45EF-B55D-D7C633E7B28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAAD6999-5678-4F24-8D2B-E16913D01515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14568" uniqueCount="2731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14587" uniqueCount="2738">
   <si>
     <t>theme</t>
   </si>
@@ -8231,6 +8231,27 @@
   </si>
   <si>
     <t>image à mettre dans énoncé</t>
+  </si>
+  <si>
+    <t>devrait etre un zip à la place du docx</t>
+  </si>
+  <si>
+    <t>manque docx ET zip</t>
+  </si>
+  <si>
+    <t>manque image à télécharger</t>
+  </si>
+  <si>
+    <t>devrait etre une image à télécharger à la place du docx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">! docx inexistant; ne devrai pas téléchargeable  ! </t>
+  </si>
+  <si>
+    <t>! docx inexistant; ne devrai pas téléchargeable  !  par contre manque la liste des mots, il faut en faire une zone de texte</t>
+  </si>
+  <si>
+    <t>! docx inexistant; ne devrai pas téléchargeable  !  Manque image à télécharger</t>
   </si>
 </sst>
 </file>
@@ -8389,7 +8410,8 @@
     </filterColumn>
     <filterColumn colId="1">
       <filters>
-        <filter val="Insérer une image"/>
+        <filter val="Insérer un tableau"/>
+        <filter val="Tableau avancé"/>
       </filters>
     </filterColumn>
     <filterColumn colId="6">
@@ -16191,7 +16213,9 @@
       <c r="G309" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="H309" s="2"/>
+      <c r="H309" s="2" t="s">
+        <v>2733</v>
+      </c>
     </row>
     <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" s="2" t="s">
@@ -16505,7 +16529,7 @@
       </c>
       <c r="H322" s="2"/>
     </row>
-    <row r="323" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A323" s="2" t="s">
         <v>404</v>
       </c>
@@ -16601,7 +16625,7 @@
       </c>
       <c r="H326" s="2"/>
     </row>
-    <row r="327" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A327" s="2" t="s">
         <v>404</v>
       </c>
@@ -16623,7 +16647,9 @@
       <c r="G327" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="H327" s="2"/>
+      <c r="H327" s="2" t="s">
+        <v>2736</v>
+      </c>
     </row>
     <row r="328" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" s="2" t="s">
@@ -16697,7 +16723,7 @@
       </c>
       <c r="H330" s="2"/>
     </row>
-    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A331" s="2" t="s">
         <v>404</v>
       </c>
@@ -16719,7 +16745,9 @@
       <c r="G331" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="H331" s="2"/>
+      <c r="H331" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" s="2" t="s">
@@ -16793,7 +16821,7 @@
       </c>
       <c r="H334" s="2"/>
     </row>
-    <row r="335" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A335" s="2" t="s">
         <v>404</v>
       </c>
@@ -16815,7 +16843,9 @@
       <c r="G335" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="H335" s="2"/>
+      <c r="H335" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" s="2" t="s">
@@ -16889,7 +16919,7 @@
       </c>
       <c r="H338" s="2"/>
     </row>
-    <row r="339" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A339" s="2" t="s">
         <v>404</v>
       </c>
@@ -16911,7 +16941,9 @@
       <c r="G339" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="H339" s="2"/>
+      <c r="H339" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="340" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" s="2" t="s">
@@ -16985,7 +17017,7 @@
       </c>
       <c r="H342" s="2"/>
     </row>
-    <row r="343" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A343" s="2" t="s">
         <v>404</v>
       </c>
@@ -17007,7 +17039,9 @@
       <c r="G343" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="H343" s="2"/>
+      <c r="H343" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="344" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" s="2" t="s">
@@ -17081,7 +17115,7 @@
       </c>
       <c r="H346" s="2"/>
     </row>
-    <row r="347" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A347" s="2" t="s">
         <v>404</v>
       </c>
@@ -17103,7 +17137,9 @@
       <c r="G347" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="H347" s="2"/>
+      <c r="H347" s="2" t="s">
+        <v>2737</v>
+      </c>
     </row>
     <row r="348" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" s="2" t="s">
@@ -17177,7 +17213,7 @@
       </c>
       <c r="H350" s="2"/>
     </row>
-    <row r="351" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A351" s="2" t="s">
         <v>404</v>
       </c>
@@ -17273,7 +17309,7 @@
       </c>
       <c r="H354" s="2"/>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A355" s="2" t="s">
         <v>404</v>
       </c>
@@ -18282,7 +18318,7 @@
       </c>
       <c r="H396" s="2"/>
     </row>
-    <row r="397" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" s="2" t="s">
         <v>404</v>
       </c>
@@ -18380,7 +18416,7 @@
       </c>
       <c r="H400" s="2"/>
     </row>
-    <row r="401" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" s="2" t="s">
         <v>404</v>
       </c>
@@ -18402,7 +18438,9 @@
       <c r="G401" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="H401" s="2"/>
+      <c r="H401" s="2" t="s">
+        <v>2731</v>
+      </c>
     </row>
     <row r="402" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" s="2" t="s">
@@ -18524,7 +18562,7 @@
       </c>
       <c r="H406" s="2"/>
     </row>
-    <row r="407" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A407" s="2" t="s">
         <v>404</v>
       </c>
@@ -18546,9 +18584,11 @@
       <c r="G407" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="H407" s="2"/>
-    </row>
-    <row r="408" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H407" s="2" t="s">
+        <v>2732</v>
+      </c>
+    </row>
+    <row r="408" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A408" s="2" t="s">
         <v>404</v>
       </c>
@@ -18570,7 +18610,9 @@
       <c r="G408" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="H408" s="2"/>
+      <c r="H408" s="2" t="s">
+        <v>2733</v>
+      </c>
     </row>
     <row r="409" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" s="2" t="s">
@@ -18644,7 +18686,7 @@
       </c>
       <c r="H411" s="2"/>
     </row>
-    <row r="412" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" s="2" t="s">
         <v>404</v>
       </c>
@@ -18666,7 +18708,9 @@
       <c r="G412" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="H412" s="2"/>
+      <c r="H412" s="2" t="s">
+        <v>2734</v>
+      </c>
     </row>
     <row r="413" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" s="2" t="s">
@@ -18716,7 +18760,7 @@
       </c>
       <c r="H414" s="2"/>
     </row>
-    <row r="415" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" s="2" t="s">
         <v>404</v>
       </c>
@@ -18738,7 +18782,9 @@
       <c r="G415" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="H415" s="2"/>
+      <c r="H415" s="2" t="s">
+        <v>2726</v>
+      </c>
     </row>
     <row r="416" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" s="2" t="s">
@@ -18812,7 +18858,7 @@
       </c>
       <c r="H418" s="2"/>
     </row>
-    <row r="419" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" s="2" t="s">
         <v>404</v>
       </c>
@@ -18834,7 +18880,9 @@
       <c r="G419" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="H419" s="2"/>
+      <c r="H419" s="2" t="s">
+        <v>2731</v>
+      </c>
     </row>
     <row r="420" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" s="2" t="s">
@@ -18932,7 +18980,7 @@
       </c>
       <c r="H423" s="2"/>
     </row>
-    <row r="424" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" s="2" t="s">
         <v>404</v>
       </c>
@@ -18954,7 +19002,9 @@
       <c r="G424" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="H424" s="2"/>
+      <c r="H424" s="2" t="s">
+        <v>2726</v>
+      </c>
     </row>
     <row r="425" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" s="2" t="s">
@@ -19028,7 +19078,7 @@
       </c>
       <c r="H427" s="2"/>
     </row>
-    <row r="428" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A428" s="2" t="s">
         <v>404</v>
       </c>
@@ -19050,7 +19100,9 @@
       <c r="G428" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="H428" s="2"/>
+      <c r="H428" s="2" t="s">
+        <v>2726</v>
+      </c>
     </row>
     <row r="429" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A429" s="2" t="s">
@@ -19100,7 +19152,7 @@
       </c>
       <c r="H430" s="2"/>
     </row>
-    <row r="431" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:8" ht="36" hidden="1" x14ac:dyDescent="0.35">
       <c r="A431" s="2" t="s">
         <v>404</v>
       </c>
@@ -19124,7 +19176,7 @@
       </c>
       <c r="H431" s="2"/>
     </row>
-    <row r="432" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" s="2" t="s">
         <v>404</v>
       </c>
@@ -19146,7 +19198,9 @@
       <c r="G432" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="H432" s="2"/>
+      <c r="H432" s="2" t="s">
+        <v>2733</v>
+      </c>
     </row>
     <row r="433" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" s="2" t="s">
@@ -20088,7 +20142,9 @@
       <c r="G471" s="2" t="s">
         <v>637</v>
       </c>
-      <c r="H471" s="2"/>
+      <c r="H471" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="472" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A472" s="2" t="s">
@@ -23762,7 +23818,7 @@
       </c>
       <c r="H624" s="2"/>
     </row>
-    <row r="625" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="625" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A625" s="2" t="s">
         <v>404</v>
       </c>
@@ -23882,7 +23938,7 @@
       </c>
       <c r="H629" s="2"/>
     </row>
-    <row r="630" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="630" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A630" s="2" t="s">
         <v>404</v>
       </c>
@@ -23904,7 +23960,9 @@
       <c r="G630" s="2" t="s">
         <v>833</v>
       </c>
-      <c r="H630" s="2"/>
+      <c r="H630" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="631" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A631" s="2" t="s">
@@ -23978,7 +24036,7 @@
       </c>
       <c r="H633" s="2"/>
     </row>
-    <row r="634" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="634" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A634" s="2" t="s">
         <v>404</v>
       </c>
@@ -24000,7 +24058,9 @@
       <c r="G634" s="2" t="s">
         <v>839</v>
       </c>
-      <c r="H634" s="2"/>
+      <c r="H634" s="2" t="s">
+        <v>2735</v>
+      </c>
     </row>
     <row r="635" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A635" s="2" t="s">
@@ -24074,7 +24134,7 @@
       </c>
       <c r="H637" s="2"/>
     </row>
-    <row r="638" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="638" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A638" s="2" t="s">
         <v>404</v>
       </c>
@@ -24170,7 +24230,7 @@
       </c>
       <c r="H641" s="2"/>
     </row>
-    <row r="642" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="642" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A642" s="2" t="s">
         <v>404</v>
       </c>
@@ -24266,7 +24326,7 @@
       </c>
       <c r="H645" s="2"/>
     </row>
-    <row r="646" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="646" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A646" s="2" t="s">
         <v>404</v>
       </c>
@@ -24362,7 +24422,7 @@
       </c>
       <c r="H649" s="2"/>
     </row>
-    <row r="650" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="650" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A650" s="2" t="s">
         <v>404</v>
       </c>
@@ -24458,7 +24518,7 @@
       </c>
       <c r="H653" s="2"/>
     </row>
-    <row r="654" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="654" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A654" s="2" t="s">
         <v>404</v>
       </c>

</xml_diff>